<commit_message>
v2.2: data quality 100%, AI capability levels (L0/L1/L2), iterative review workflow, README overhaul
</commit_message>
<xml_diff>
--- a/Extract/TXCrawl_result.xlsx
+++ b/Extract/TXCrawl_result.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I20"/>
+  <dimension ref="A1:I25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1480,6 +1480,191 @@
         </is>
       </c>
     </row>
+    <row r="21">
+      <c r="A21" t="n">
+        <v>42</v>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>腾讯研究院AI速递 20260423</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>OpenAI发布ChatGPT Images 2.0支持复杂视觉任务和高密度文本渲染，最高2K分辨率，首次引入思考能力可联网获取实时信息；Anthropic推出STEM Fellow项目招募各学科专家驻场旧金山校准Claude输出；谷歌发布Deep Research智能体支持MCP协议与原生图表</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>https://www.sohu.com/a/1013204317_455313</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>2026.04.23</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr"/>
+      <c r="G21" t="inlineStr"/>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>ChatGPT Images 2.0（OpenAI）、Claude Code（Anthropic）、Deep Research / Deep Research Max（谷歌）、Gemini 3.1 Pro（谷歌）、Codex（OpenAI）、Sage（商汤绝影）、NeuroVLA（智平方+港科大）、Reflection（开源）</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>ChatGPT Images 2.0、Deep Research / Deep Research Max、Sage、NeuroVLA</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="n">
+        <v>43</v>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>腾讯研究院AI速递 20260422</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>GPT-Image-2全量开放，精准生成中文试卷、书法和报纸排版，彻底解决AI生图中文乱码问题；Codex上线Chronicle功能通过屏幕上下文形成记忆；谷歌组攻坚队追赶Anthropic，布林亲自督战Claude</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>https://www.sohu.com/a/1012691881_455313</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>2026.04.22</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr"/>
+      <c r="G22" t="inlineStr"/>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>GPT Image 2（OpenAI）、Codex（OpenAI）、Claude Code（Anthropic）、Kimi K2.6（月之暗面）、miclaw（小米）、QClaw（腾讯）</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>GPT Image 2、QClaw</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>44</v>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>腾讯研究院AI速递 20260421</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>OpenAI静默升级GPT Pro速度翻4倍，GPT-5.4在视觉理解与前端代码生成上接近质变；代号Spud的GPT-5.5或已完成预训练预计Q2发布</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>https://www.sohu.com/a/1012194989_455313</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>2026.04.21</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr"/>
+      <c r="G23" t="inlineStr"/>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>GPT-5.4（OpenAI）、GPT-5.5/Spud（OpenAI）、Qwen3.6-Max-Preview（阿里）、Claude Mythos（Anthropic）、闪应用（灵光）、OmniHand 3 Ultra-T / Lite（临界点）</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>GPT-5.5、Qwen3.6-Max-Preview、Claude Mythos、闪应用、OmniHand 3 Ultra-T、OmniHand 3 Lite</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="n">
+        <v>45</v>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>腾讯研究院AI速递 20260420</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>OpenAI新生图模型GPT Image 2在LM Arena短暂泄露，文字渲染、指令跟随、真实感和世界知识四维度均超越Nano Banana Pro；Anthropic推出Claude Design，Figma股价下跌</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>https://www.sohu.com/a/1011735544_455313</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>2026.04.20</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr"/>
+      <c r="G24" t="inlineStr"/>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>GPT Image 2（OpenAI）、Nano Banana Pro（谷歌）、Claude Design（Anthropic）、Claude Opus 4.7（Anthropic）、AutoClaw（智谱）、π0.7（Physical Intelligence）、ABot-World / ABot-M / ABot-N / ABot-Claw（高德）、GPT-Rosalind（OpenAI）、Veo 3.1（谷歌）</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>Claude Design、π0.7、ABot-World、ABot-M、ABot-N、ABot-Claw、GPT-Rosalind、Veo 3.1</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="n">
+        <v>46</v>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>腾讯研究院AI速递 20260417</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Anthropic发布Claude Opus 4.7定价与4.6相同，新增自我验证能力，Rakuten生产任务解决率提升3倍；视觉能力大幅增强支持最高375万像素图像输入；OpenAI重写Agents SDK打造生产级Agent底座</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>https://www.sohu.com/a/1010572967_455313</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>2026.04.17</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr"/>
+      <c r="G25" t="inlineStr"/>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>Claude Opus 4.7（Anthropic）、Nano Banana 2 / Gemini 3.1 Flash Image（谷歌）、Gemini 3.1 Flash TTS（谷歌）、混元3D世界模型2.0（腾讯）、HappyOyster（阿里）、StepAudio 2.5 TTS（阶跃星辰）、LingBot-Map（蚂蚁）、MaxHermes（MiniMax）</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>Nano Banana 2、混元3D世界模型2.0、HappyOyster、StepAudio 2.5 TTS、LingBot-Map、MaxHermes</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>